<commit_message>
Add SOH report for 2026-10-07
</commit_message>
<xml_diff>
--- a/reports/SOH_06_10_2026.xlsx
+++ b/reports/SOH_06_10_2026.xlsx
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>-18</v>
+        <v>8</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>21000</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>25000</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>249</v>
+        <v>272</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1100</v>
+        <v>1129</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>40000</v>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>10500</v>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>40000</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>469</v>
+        <v>486</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>10500</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>48000</v>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>24000</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>385</v>
+        <v>367</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>10500</v>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>21000</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>635</v>
+        <v>629</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1080</v>
+        <v>1076</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="E48" s="3" t="n">
         <v>18000</v>
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>81000</v>
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="E50" s="3" t="n">
         <v>81000</v>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>81000</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>560</v>
+        <v>550</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>336</v>
+        <v>319</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>26500</v>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E61" s="3" t="n">
         <v>3900</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>824</v>
+        <v>811</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E63" s="3" t="n">
         <v>26500</v>
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>26500</v>
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E67" s="3" t="n">
         <v>51000</v>
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="E68" s="3" t="n">
         <v>26500</v>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E70" s="3" t="n">
         <v>51000</v>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>977</v>
+        <v>942</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>3000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>774</v>
+        <v>758</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>3000</v>
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>-26</v>
+        <v>0</v>
       </c>
       <c r="E84" s="3" t="n">
         <v>9000</v>
@@ -2813,7 +2813,7 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E85" s="3" t="n">
         <v>20000</v>
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E86" s="3" t="n">
         <v>20000</v>
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E87" s="3" t="n">
         <v>30000</v>
@@ -2897,7 +2897,7 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E88" s="3" t="n">
         <v>30000</v>
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E89" s="3" t="n">
         <v>31000</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>829</v>
+        <v>805</v>
       </c>
       <c r="E93" s="3" t="n">
         <v>8000</v>
@@ -3065,7 +3065,7 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E94" s="3" t="n">
         <v>21000</v>
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E96" s="3" t="n">
         <v>8000</v>
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="E98" s="3" t="n">
         <v>8597</v>
@@ -3205,7 +3205,7 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E99" s="3" t="n">
         <v>8597</v>
@@ -3233,7 +3233,7 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="E100" s="3" t="n">
         <v>8597</v>
@@ -3261,7 +3261,7 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E101" s="3" t="n">
         <v>8597</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>4708</v>
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E103" s="3" t="n">
         <v>4708</v>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E104" s="3" t="n">
         <v>4708</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E105" s="3" t="n">
         <v>4708</v>
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E106" s="3" t="n">
         <v>12500</v>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E108" s="3" t="n">
         <v>1</v>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>2828</v>
+        <v>2892</v>
       </c>
       <c r="E109" s="3" t="n">
         <v>3876</v>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>2633</v>
+        <v>2691</v>
       </c>
       <c r="E110" s="3" t="n">
         <v>3500</v>
@@ -3541,7 +3541,7 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E111" s="3" t="n">
         <v>25000</v>
@@ -3569,7 +3569,7 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="E112" s="3" t="n">
         <v>25000</v>
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E113" s="3" t="n">
         <v>25000</v>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E114" s="3" t="n">
         <v>36000</v>
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E115" s="3" t="n">
         <v>36000</v>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="E116" s="3" t="n">
         <v>36000</v>
@@ -3709,7 +3709,7 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E117" s="3" t="n">
         <v>5000</v>
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="E118" s="3" t="n">
         <v>5000</v>
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E119" s="3" t="n">
         <v>5000</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2241</v>
+        <v>2207</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>4878</v>
+        <v>4801</v>
       </c>
       <c r="E126" s="3" t="n">
         <v>2500</v>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>730</v>
+        <v>384</v>
       </c>
       <c r="E128" s="3" t="n">
         <v>3500</v>
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
       <c r="E129" s="3" t="n">
         <v>2500</v>
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>-25</v>
+        <v>0</v>
       </c>
       <c r="E130" s="3" t="n">
         <v>3500</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>355</v>
+        <v>163</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>454</v>
+        <v>0</v>
       </c>
       <c r="E137" s="3" t="n">
         <v>3500</v>
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E156" s="3" t="n">
         <v>26000</v>
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="E159" s="3" t="n">
         <v>1</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>491</v>
+        <v>445</v>
       </c>
       <c r="E174" s="3" t="n">
         <v>13500</v>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E177" s="3" t="n">
         <v>1</v>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -6953,7 +6953,7 @@
         </is>
       </c>
       <c r="D236" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E236" s="3" t="n">
         <v>6750</v>
@@ -9654,7 +9654,7 @@
         </is>
       </c>
       <c r="D333" s="2" t="n">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="E333" s="3" t="n">
         <v>5000</v>
@@ -9682,7 +9682,7 @@
         </is>
       </c>
       <c r="D334" s="2" t="n">
-        <v>523</v>
+        <v>537</v>
       </c>
       <c r="E334" s="3" t="n">
         <v>2500</v>
@@ -16402,7 +16402,7 @@
         </is>
       </c>
       <c r="D574" s="2" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="E574" s="3" t="n">
         <v>39521</v>
@@ -20491,7 +20491,7 @@
         </is>
       </c>
       <c r="D720" s="2" t="n">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="E720" s="3" t="n">
         <v>8782</v>
@@ -29597,7 +29597,7 @@
         </is>
       </c>
       <c r="D1045" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E1045" s="3" t="n">
         <v>11977</v>
@@ -33741,7 +33741,7 @@
         </is>
       </c>
       <c r="D1193" s="2" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E1193" s="3" t="n">
         <v>52044</v>
@@ -34161,7 +34161,7 @@
         </is>
       </c>
       <c r="D1208" s="2" t="n">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="E1208" s="3" t="n">
         <v>24420</v>
@@ -34553,7 +34553,7 @@
         </is>
       </c>
       <c r="D1222" s="2" t="n">
-        <v>85</v>
+        <v>37</v>
       </c>
       <c r="E1222" s="3" t="n">
         <v>32769</v>
@@ -38529,7 +38529,7 @@
         </is>
       </c>
       <c r="D1364" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E1364" s="3" t="n">
         <v>18059</v>

</xml_diff>